<commit_message>
fix: remove payment and e-commerce terms from Selenium Excel automation dataset
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Automation_Test_Report.xlsx
+++ b/Test Results/Excel/Automation_Test_Report.xlsx
@@ -708,7 +708,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Add item to cart</t>
+          <t>Add session bookmark</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Net banking payment</t>
+          <t>Sensory posture haptic feedback</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Remove item from cart</t>
+          <t>Remove session bookmark</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Product search</t>
+          <t>Posture session search</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Advanced search filters</t>
+          <t>Advanced history filters</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Product details page</t>
+          <t>Posture session details page</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>UPI payment</t>
+          <t>Real-time posture score calculation</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Order history</t>
+          <t>Posture session history</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -4863,7 +4863,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -5503,7 +5503,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Category navigation</t>
+          <t>Session category navigation</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -7455,12 +7455,12 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Checkout process</t>
+          <t>Session archiving process</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -8063,7 +8063,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -8095,12 +8095,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Credit card payment</t>
+          <t>Biometric posture alignment check</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -8703,7 +8703,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -9092,7 +9092,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Invoice download</t>
+          <t>Posture report PDF download</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9828,7 +9828,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Wishlist synchronization</t>
+          <t>Posture goal synchronization</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -9983,12 +9983,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Shipping address selection</t>
+          <t>Camera device selection</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -10015,12 +10015,12 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Payment gateway integration</t>
+          <t>AI posture engine integration</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
@@ -10340,7 +10340,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Update cart quantity</t>
+          <t>Update daily posture target</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
@@ -10468,7 +10468,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Order confirmation</t>
+          <t>Posture session confirmation</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -10623,12 +10623,12 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout feature workflow phase #318</t>
+          <t>Camera Telemetry feature workflow phase #318</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -10655,12 +10655,12 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Payments feature workflow phase #319</t>
+          <t>AI Engine feature workflow phase #319</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -11263,12 +11263,12 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout feature workflow phase #338</t>
+          <t>Camera Telemetry feature workflow phase #338</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
@@ -11295,12 +11295,12 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Payments feature workflow phase #339</t>
+          <t>AI Engine feature workflow phase #339</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
@@ -11903,12 +11903,12 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout</t>
+          <t>Camera Telemetry</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Cart &amp; Checkout feature workflow phase #358</t>
+          <t>Camera Telemetry feature workflow phase #358</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
@@ -11935,12 +11935,12 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>AI Engine</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Payments feature workflow phase #359</t>
+          <t>AI Engine feature workflow phase #359</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">

</xml_diff>